<commit_message>
fix(contracts): polish catalog import workbook UX
</commit_message>
<xml_diff>
--- a/docs/catalog-import/catalog-import-v1-template.xlsx
+++ b/docs/catalog-import/catalog-import-v1-template.xlsx
@@ -14,344 +14,419 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="158">
+  <si>
+    <t>批次内关联 ID【必填】</t>
+  </si>
+  <si>
+    <t>来源 ID【必填】</t>
+  </si>
+  <si>
+    <t>平台目录 ID【更新时填】</t>
+  </si>
+  <si>
+    <t>题名【必填】</t>
+  </si>
+  <si>
+    <t>类别【必填】</t>
+  </si>
+  <si>
+    <t>朝代</t>
+  </si>
+  <si>
+    <t>朝代状态</t>
+  </si>
+  <si>
+    <t>年代文本</t>
+  </si>
+  <si>
+    <t>年代状态</t>
+  </si>
+  <si>
+    <t>省级行政区</t>
+  </si>
+  <si>
+    <t>省级状态</t>
+  </si>
+  <si>
+    <t>地市级行政区</t>
+  </si>
+  <si>
+    <t>地市状态</t>
+  </si>
+  <si>
+    <t>区县级行政区</t>
+  </si>
+  <si>
+    <t>区县状态</t>
+  </si>
+  <si>
+    <t>当前地点</t>
+  </si>
+  <si>
+    <t>地点状态</t>
+  </si>
+  <si>
+    <t>当前保管机构</t>
+  </si>
+  <si>
+    <t>保管状态</t>
+  </si>
+  <si>
+    <t>描述</t>
+  </si>
+  <si>
+    <t>描述状态</t>
+  </si>
+  <si>
+    <t>内部备注</t>
+  </si>
+  <si>
+    <t>catalogImportId</t>
+  </si>
+  <si>
+    <t>sourceId</t>
+  </si>
+  <si>
+    <t>catalogId</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>catalogKind</t>
+  </si>
+  <si>
+    <t>dynasty</t>
+  </si>
+  <si>
+    <t>dynastyState</t>
+  </si>
+  <si>
+    <t>dateText</t>
+  </si>
+  <si>
+    <t>dateTextState</t>
+  </si>
+  <si>
+    <t>province</t>
+  </si>
+  <si>
+    <t>provinceState</t>
+  </si>
+  <si>
+    <t>prefecture</t>
+  </si>
+  <si>
+    <t>prefectureState</t>
+  </si>
+  <si>
+    <t>county</t>
+  </si>
+  <si>
+    <t>countyState</t>
+  </si>
+  <si>
+    <t>currentLocation</t>
+  </si>
+  <si>
+    <t>currentLocationState</t>
+  </si>
+  <si>
+    <t>currentCustodian</t>
+  </si>
+  <si>
+    <t>currentCustodianState</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>descriptionState</t>
+  </si>
+  <si>
+    <t>ownerNote</t>
+  </si>
+  <si>
+    <t>别名【必填】</t>
+  </si>
+  <si>
+    <t>别名类型【必填】</t>
+  </si>
+  <si>
+    <t>alias</t>
+  </si>
+  <si>
+    <t>aliasType</t>
+  </si>
+  <si>
+    <t>来源题名</t>
+  </si>
+  <si>
+    <t>原始来源类型</t>
+  </si>
+  <si>
+    <t>来源链接</t>
+  </si>
+  <si>
+    <t>来源备注</t>
+  </si>
+  <si>
+    <t>sourceTitle</t>
+  </si>
+  <si>
+    <t>sourceTypeRaw</t>
+  </si>
+  <si>
+    <t>sourceUrl</t>
+  </si>
+  <si>
+    <t>sourceNote</t>
+  </si>
+  <si>
+    <t>摩崖目录导入模板 — Owner 使用说明</t>
+  </si>
+  <si>
+    <t>本文件是 Owner / Editor working template；PostgreSQL 才是 canonical runtime source of truth。请复制模板后填写具体 batch，不要直接编辑正式模板。</t>
+  </si>
+  <si>
+    <t>A. Owner 快速开始</t>
+  </si>
+  <si>
+    <t>1. 复制本模板，建立一个具体 batch workbook；不要直接修改正式模板。</t>
+  </si>
+  <si>
+    <t>2. 新建 Catalog：catalogId 留空；更新 Catalog：catalogId 必须填写既有且不可变的目标 ID。</t>
+  </si>
+  <si>
+    <t>3. 每条 01_Catalog 都要填写 catalogImportId、sourceId、title、catalogKind。</t>
+  </si>
+  <si>
+    <t>4. 子表用 catalogImportId 关联 01_Catalog；catalogImportId ≠ sourceId ≠ catalogId。</t>
+  </si>
+  <si>
+    <t>5. value 有内容时，state 留空或选 VALUE；state 的英文 machine value 不翻译。</t>
+  </si>
+  <si>
+    <t>6. blank 或 UNSUPPLIED 表示本批次未提供；UNKNOWN 表示未知；NOT_APPLICABLE 表示不适用。</t>
+  </si>
+  <si>
+    <t>7. CLEAR 才表示请求清除，并需要逐字段审批；blank ≠ delete。</t>
+  </si>
+  <si>
+    <t>8. aliasType 只允许 alternate / historical；CatalogKind 只允许 inscription / calligraphy。</t>
+  </si>
+  <si>
+    <t>9. duplicate 只产生候选，不自动 merge、改写 CatalogId 或解除 blocker。</t>
+  </si>
+  <si>
+    <t>10. 成功 Import ≠ Publish；导入不改变 publication lifecycle。</t>
+  </si>
+  <si>
+    <t>B. Identity / State / Location guidance</t>
+  </si>
+  <si>
+    <t>Identity：catalogImportId 是 batch-local 关联键；sourceId 是来源记录身份；catalogId 是 Catalog 身份。三者不可互换。CatalogId / SourceId linkage conflict 不可审批、不可 Apply。</t>
+  </si>
+  <si>
+    <t>State：事实字段使用 VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR；description 仅使用 VALUE / UNSUPPLIED / CLEAR。state 为 UNKNOWN、NOT_APPLICABLE 或 CLEAR 时，value 必须为空。</t>
+  </si>
+  <si>
+    <t>Location：province / prefecture / county 是行政区；currentLocation 是具体地点或遗址；currentCustodian 是当前管理或保管机构。</t>
+  </si>
+  <si>
+    <t>纯 synthetic 示例：province=福建省，prefecture=泉州市，county=洛江区，currentLocation=万安某处，currentCustodian=某文物管理机构。该示例不是 production data。</t>
+  </si>
+  <si>
+    <t>SourceId mirroring：03_Provenance 可在相同 catalogImportId 下镜像主表 sourceId 以扩展同一 SourceRecord metadata；重复 pair 或跨 Catalog 绑定冲突会失败。</t>
+  </si>
+  <si>
+    <t>C. Field Guide</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>中文名称</t>
+  </si>
+  <si>
+    <t>Machine header</t>
+  </si>
+  <si>
+    <t>Requiredness</t>
+  </si>
+  <si>
+    <t>如何填写</t>
+  </si>
+  <si>
+    <t>示例</t>
+  </si>
+  <si>
+    <t>01_Catalog</t>
+  </si>
   <si>
     <t>批次内关联 ID</t>
   </si>
   <si>
+    <t>必填</t>
+  </si>
+  <si>
+    <t>同一批次内关联主表与子表；不是 Catalog 的永久身份。</t>
+  </si>
+  <si>
+    <t>synthetic-item-001</t>
+  </si>
+  <si>
     <t>来源 ID</t>
   </si>
   <si>
-    <t>Catalog ID（更新）</t>
+    <t>来源记录身份；不得与 catalogId 混用。</t>
+  </si>
+  <si>
+    <t>synthetic-source-001</t>
+  </si>
+  <si>
+    <t>平台目录 ID</t>
+  </si>
+  <si>
+    <t>更新时填</t>
+  </si>
+  <si>
+    <t>新建时留空；更新时填写不可变的既有 Catalog 目标。</t>
+  </si>
+  <si>
+    <t>synthetic-catalog-001</t>
   </si>
   <si>
     <t>题名</t>
   </si>
   <si>
-    <t>目录类型</t>
-  </si>
-  <si>
-    <t>朝代</t>
-  </si>
-  <si>
-    <t>朝代状态</t>
-  </si>
-  <si>
-    <t>年代文本</t>
-  </si>
-  <si>
-    <t>年代状态</t>
-  </si>
-  <si>
-    <t>省级行政区</t>
-  </si>
-  <si>
-    <t>省级状态</t>
-  </si>
-  <si>
-    <t>地市级行政区</t>
-  </si>
-  <si>
-    <t>地市状态</t>
-  </si>
-  <si>
-    <t>区县级行政区</t>
-  </si>
-  <si>
-    <t>区县状态</t>
-  </si>
-  <si>
-    <t>当前地点</t>
-  </si>
-  <si>
-    <t>地点状态</t>
-  </si>
-  <si>
-    <t>当前保管机构</t>
-  </si>
-  <si>
-    <t>保管状态</t>
-  </si>
-  <si>
-    <t>描述</t>
-  </si>
-  <si>
-    <t>描述状态</t>
-  </si>
-  <si>
-    <t>Owner 内部备注</t>
-  </si>
-  <si>
-    <t>catalogImportId</t>
-  </si>
-  <si>
-    <t>sourceId</t>
-  </si>
-  <si>
-    <t>catalogId</t>
-  </si>
-  <si>
-    <t>title</t>
-  </si>
-  <si>
-    <t>catalogKind</t>
-  </si>
-  <si>
-    <t>dynasty</t>
-  </si>
-  <si>
-    <t>dynastyState</t>
-  </si>
-  <si>
-    <t>dateText</t>
-  </si>
-  <si>
-    <t>dateTextState</t>
-  </si>
-  <si>
-    <t>province</t>
-  </si>
-  <si>
-    <t>provinceState</t>
-  </si>
-  <si>
-    <t>prefecture</t>
-  </si>
-  <si>
-    <t>prefectureState</t>
-  </si>
-  <si>
-    <t>county</t>
-  </si>
-  <si>
-    <t>countyState</t>
-  </si>
-  <si>
-    <t>currentLocation</t>
-  </si>
-  <si>
-    <t>currentLocationState</t>
-  </si>
-  <si>
-    <t>currentCustodian</t>
-  </si>
-  <si>
-    <t>currentCustodianState</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>descriptionState</t>
-  </si>
-  <si>
-    <t>ownerNote</t>
+    <t>条目的主要题名。</t>
+  </si>
+  <si>
+    <t>合成示例题名</t>
+  </si>
+  <si>
+    <t>类别</t>
+  </si>
+  <si>
+    <t>只选择 inscription 或 calligraphy。</t>
+  </si>
+  <si>
+    <t>inscription</t>
+  </si>
+  <si>
+    <t>选填</t>
+  </si>
+  <si>
+    <t>原始事实文本；与右侧状态配对。</t>
+  </si>
+  <si>
+    <t>唐（synthetic）</t>
+  </si>
+  <si>
+    <t>留空等同 UNSUPPLIED；blank 不删除。</t>
+  </si>
+  <si>
+    <t>VALUE</t>
+  </si>
+  <si>
+    <t>不规范化的年代描述；与右侧状态配对。</t>
+  </si>
+  <si>
+    <t>贞观年间（synthetic）</t>
+  </si>
+  <si>
+    <t>VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR。</t>
+  </si>
+  <si>
+    <t>行政区事实，例如“福建省”；不是地点名称。</t>
+  </si>
+  <si>
+    <t>福建省（synthetic）</t>
+  </si>
+  <si>
+    <t>与省级行政区配对。</t>
+  </si>
+  <si>
+    <t>行政区事实，例如“泉州市”。</t>
+  </si>
+  <si>
+    <t>泉州市（synthetic）</t>
+  </si>
+  <si>
+    <t>与地市级行政区配对。</t>
+  </si>
+  <si>
+    <t>行政区事实，例如“洛江区”。</t>
+  </si>
+  <si>
+    <t>洛江区（synthetic）</t>
+  </si>
+  <si>
+    <t>与区县级行政区配对。</t>
+  </si>
+  <si>
+    <t>具体地点或遗址名称，例如“万安某处（synthetic）”。</t>
+  </si>
+  <si>
+    <t>万安某处（synthetic）</t>
+  </si>
+  <si>
+    <t>与当前地点配对。</t>
+  </si>
+  <si>
+    <t>管理或保管主体；不是行政区或地点。</t>
+  </si>
+  <si>
+    <t>某文物管理机构（synthetic）</t>
+  </si>
+  <si>
+    <t>与当前保管机构配对。</t>
+  </si>
+  <si>
+    <t>描述文本；状态仅允许 VALUE / UNSUPPLIED / CLEAR。</t>
+  </si>
+  <si>
+    <t>纯合成描述示例</t>
+  </si>
+  <si>
+    <t>blank 不删除；CLEAR 会进入逐字段审批。</t>
+  </si>
+  <si>
+    <t>仅供 Owner 审核；不发布，不提供 destructive state。</t>
+  </si>
+  <si>
+    <t>纯合成内部备注</t>
+  </si>
+  <si>
+    <t>02_Aliases</t>
+  </si>
+  <si>
+    <t>子表行必填</t>
+  </si>
+  <si>
+    <t>必须指向 01_Catalog 的 catalogImportId。</t>
   </si>
   <si>
     <t>别名</t>
   </si>
   <si>
+    <t>完整的别名文本。</t>
+  </si>
+  <si>
+    <t>合成示例别名</t>
+  </si>
+  <si>
     <t>别名类型</t>
   </si>
   <si>
-    <t>alias</t>
-  </si>
-  <si>
-    <t>aliasType</t>
-  </si>
-  <si>
-    <t>来源题名</t>
-  </si>
-  <si>
-    <t>原始来源类型</t>
-  </si>
-  <si>
-    <t>来源链接</t>
-  </si>
-  <si>
-    <t>来源备注</t>
-  </si>
-  <si>
-    <t>sourceTitle</t>
-  </si>
-  <si>
-    <t>sourceTypeRaw</t>
-  </si>
-  <si>
-    <t>sourceUrl</t>
-  </si>
-  <si>
-    <t>sourceNote</t>
-  </si>
-  <si>
-    <t>摩崖目录导入模板 — Owner 使用说明</t>
-  </si>
-  <si>
-    <t>本文件是 Owner / Editor working template；PostgreSQL 才是 canonical runtime source of truth。请复制模板后填写具体 batch，不要直接编辑正式模板。</t>
-  </si>
-  <si>
-    <t>A. Owner 快速开始</t>
-  </si>
-  <si>
-    <t>1. 复制本模板，建立一个具体 batch workbook；不要直接修改正式模板。</t>
-  </si>
-  <si>
-    <t>2. 新建 Catalog：catalogId 留空；更新 Catalog：catalogId 必须填写既有且不可变的目标 ID。</t>
-  </si>
-  <si>
-    <t>3. 每条 01_Catalog 都要填写 catalogImportId、sourceId、title、catalogKind。</t>
-  </si>
-  <si>
-    <t>4. 子表用 catalogImportId 关联 01_Catalog；catalogImportId ≠ sourceId ≠ catalogId。</t>
-  </si>
-  <si>
-    <t>5. value 有内容时，state 留空或选 VALUE；state 的英文 machine value 不翻译。</t>
-  </si>
-  <si>
-    <t>6. blank 或 UNSUPPLIED 表示本批次未提供；UNKNOWN 表示未知；NOT_APPLICABLE 表示不适用。</t>
-  </si>
-  <si>
-    <t>7. CLEAR 才表示请求清除，并需要逐字段审批；blank ≠ delete。</t>
-  </si>
-  <si>
-    <t>8. aliasType 只允许 alternate / historical；CatalogKind 只允许 inscription / calligraphy。</t>
-  </si>
-  <si>
-    <t>9. duplicate 只产生候选，不自动 merge、改写 CatalogId 或解除 blocker。</t>
-  </si>
-  <si>
-    <t>10. 成功 Import ≠ Publish；导入不改变 publication lifecycle。</t>
-  </si>
-  <si>
-    <t>B. Identity / State / Location guidance</t>
-  </si>
-  <si>
-    <t>Identity：catalogImportId 是 batch-local 关联键；sourceId 是来源记录身份；catalogId 是 Catalog 身份。三者不可互换。CatalogId / SourceId linkage conflict 不可审批、不可 Apply。</t>
-  </si>
-  <si>
-    <t>State：事实字段使用 VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR；description 仅使用 VALUE / UNSUPPLIED / CLEAR。state 为 UNKNOWN、NOT_APPLICABLE 或 CLEAR 时，value 必须为空。</t>
-  </si>
-  <si>
-    <t>Location：province / prefecture / county 是行政区；currentLocation 是具体地点或遗址；currentCustodian 是当前管理或保管机构。</t>
-  </si>
-  <si>
-    <t>纯 synthetic 示例：province=福建省，prefecture=泉州市，county=洛江区，currentLocation=万安某处，currentCustodian=某文物管理机构。该示例不是 production data。</t>
-  </si>
-  <si>
-    <t>SourceId mirroring：03_Provenance 可在相同 catalogImportId 下镜像主表 sourceId 以扩展同一 SourceRecord metadata；重复 pair 或跨 Catalog 绑定冲突会失败。</t>
-  </si>
-  <si>
-    <t>C. Field Guide</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>中文列名</t>
-  </si>
-  <si>
-    <t>Machine header</t>
-  </si>
-  <si>
-    <t>Requiredness</t>
-  </si>
-  <si>
-    <t>说明</t>
-  </si>
-  <si>
-    <t>01_Catalog</t>
-  </si>
-  <si>
-    <t>REQUIRED</t>
-  </si>
-  <si>
-    <t>同一批次内关联主表与子表；不是 Catalog 的永久身份。</t>
-  </si>
-  <si>
-    <t>来源记录身份；不得与 catalogId 混用。</t>
-  </si>
-  <si>
-    <t>UPDATE_ONLY</t>
-  </si>
-  <si>
-    <t>新建时留空；更新时填写不可变的既有 Catalog 目标。</t>
-  </si>
-  <si>
-    <t>条目的主要题名。</t>
-  </si>
-  <si>
-    <t>只选择 inscription 或 calligraphy。</t>
-  </si>
-  <si>
-    <t>OPTIONAL</t>
-  </si>
-  <si>
-    <t>原始事实文本；与右侧状态配对。</t>
-  </si>
-  <si>
-    <t>留空等同 UNSUPPLIED；blank 不删除。</t>
-  </si>
-  <si>
-    <t>不规范化的年代描述；与右侧状态配对。</t>
-  </si>
-  <si>
-    <t>VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR。</t>
-  </si>
-  <si>
-    <t>行政区事实，例如“福建省”；不是地点名称。</t>
-  </si>
-  <si>
-    <t>与省级行政区配对。</t>
-  </si>
-  <si>
-    <t>行政区事实，例如“泉州市”。</t>
-  </si>
-  <si>
-    <t>与地市级行政区配对。</t>
-  </si>
-  <si>
-    <t>行政区事实，例如“洛江区”。</t>
-  </si>
-  <si>
-    <t>与区县级行政区配对。</t>
-  </si>
-  <si>
-    <t>具体地点或遗址名称，例如“万安某处（synthetic）”。</t>
-  </si>
-  <si>
-    <t>与当前地点配对。</t>
-  </si>
-  <si>
-    <t>管理或保管主体；不是行政区或地点。</t>
-  </si>
-  <si>
-    <t>与当前保管机构配对。</t>
-  </si>
-  <si>
-    <t>描述文本；状态仅允许 VALUE / UNSUPPLIED / CLEAR。</t>
-  </si>
-  <si>
-    <t>blank 不删除；CLEAR 会进入逐字段审批。</t>
-  </si>
-  <si>
-    <t>仅供 Owner 审核；不发布，不提供 destructive state。</t>
-  </si>
-  <si>
-    <t>02_Aliases</t>
-  </si>
-  <si>
-    <t>CHILD_ROW_REQUIRED</t>
-  </si>
-  <si>
-    <t>必须指向 01_Catalog 的 catalogImportId。</t>
-  </si>
-  <si>
-    <t>完整的别名文本。</t>
-  </si>
-  <si>
     <t>只选择 alternate 或 historical。</t>
   </si>
   <si>
+    <t>alternate</t>
+  </si>
+  <si>
     <t>03_Provenance</t>
   </si>
   <si>
@@ -361,13 +436,25 @@
     <t>来源材料的原始题名。</t>
   </si>
   <si>
+    <t>合成示例来源</t>
+  </si>
+  <si>
     <t>修剪、限长的 raw metadata；不是规范化 taxonomy。</t>
   </si>
   <si>
+    <t>地方旧志（synthetic）</t>
+  </si>
+  <si>
     <t>如填写，必须是完整 URL。</t>
   </si>
   <si>
+    <t>https://example.invalid</t>
+  </si>
+  <si>
     <t>附加 raw provenance 备注。</t>
+  </si>
+  <si>
+    <t>纯合成来源备注</t>
   </si>
   <si>
     <t>D. Advanced persistence / approval / hash notes</t>
@@ -1377,7 +1464,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr defaultRowHeight="20" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1588,7 +1675,7 @@
       <c r="E25" s="11"/>
       <c r="F25" s="11"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
         <v>76</v>
       </c>
@@ -1604,95 +1691,113 @@
       <c r="E26" s="13" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="27" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>22</v>
       </c>
       <c r="D27" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="E27" s="14" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>81</v>
-      </c>
       <c r="B28" s="15" t="s">
-        <v>1</v>
+        <v>87</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>23</v>
       </c>
       <c r="D28" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="E28" s="15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
-        <v>81</v>
-      </c>
       <c r="B29" s="14" t="s">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="C29" s="14" t="s">
         <v>24</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="30" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>3</v>
+        <v>94</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>25</v>
       </c>
       <c r="D30" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="E30" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
-        <v>81</v>
-      </c>
       <c r="B31" s="14" t="s">
-        <v>4</v>
+        <v>97</v>
       </c>
       <c r="C31" s="14" t="s">
         <v>26</v>
       </c>
       <c r="D31" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="15" t="s">
         <v>82</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="32" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
-        <v>81</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>5</v>
@@ -1701,15 +1806,18 @@
         <v>27</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="33" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>6</v>
@@ -1718,15 +1826,18 @@
         <v>28</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="34" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>7</v>
@@ -1735,15 +1846,18 @@
         <v>29</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="35" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>8</v>
@@ -1752,15 +1866,18 @@
         <v>30</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>9</v>
@@ -1769,15 +1886,18 @@
         <v>31</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="37" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>10</v>
@@ -1786,15 +1906,18 @@
         <v>32</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>11</v>
@@ -1803,15 +1926,18 @@
         <v>33</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="39" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>12</v>
@@ -1820,15 +1946,18 @@
         <v>34</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="40" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>13</v>
@@ -1837,15 +1966,18 @@
         <v>35</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="41" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>14</v>
@@ -1854,15 +1986,18 @@
         <v>36</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="42" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="42" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>15</v>
@@ -1871,15 +2006,18 @@
         <v>37</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="43" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>16</v>
@@ -1888,15 +2026,18 @@
         <v>38</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="44" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="F43" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>17</v>
@@ -1905,15 +2046,18 @@
         <v>39</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="45" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>18</v>
@@ -1922,15 +2066,18 @@
         <v>40</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="46" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+      <c r="F45" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>19</v>
@@ -1939,15 +2086,18 @@
         <v>41</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="47" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+      <c r="F46" s="15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>20</v>
@@ -1956,15 +2106,18 @@
         <v>42</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="48" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+      <c r="F47" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="48" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B48" s="15" t="s">
         <v>21</v>
@@ -1973,100 +2126,118 @@
         <v>43</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="49" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="C49" s="14" t="s">
         <v>22</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="50" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="50" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>44</v>
+        <v>131</v>
       </c>
       <c r="C50" s="15" t="s">
         <v>46</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="51" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+      <c r="F50" s="15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>45</v>
+        <v>134</v>
       </c>
       <c r="C51" s="14" t="s">
         <v>47</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="52" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="C52" s="15" t="s">
         <v>22</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="53" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+      <c r="F52" s="15" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>1</v>
+        <v>87</v>
       </c>
       <c r="C53" s="14" t="s">
         <v>23</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="54" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="54" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>48</v>
@@ -2075,15 +2246,18 @@
         <v>52</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="55" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="F54" s="15" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>49</v>
@@ -2092,15 +2266,18 @@
         <v>53</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="56" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B56" s="15" t="s">
         <v>50</v>
@@ -2109,15 +2286,18 @@
         <v>54</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="57" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+      <c r="F56" s="15" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="57" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>51</v>
@@ -2126,15 +2306,18 @@
         <v>55</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>117</v>
+        <v>145</v>
+      </c>
+      <c r="F57" s="14" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="61" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="11" t="s">
-        <v>118</v>
+        <v>147</v>
       </c>
       <c r="B61" s="11"/>
       <c r="C61" s="11"/>
@@ -2144,7 +2327,7 @@
     </row>
     <row r="62" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="12" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="B62" s="12"/>
       <c r="C62" s="12"/>
@@ -2154,7 +2337,7 @@
     </row>
     <row r="63" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="12"/>
@@ -2164,7 +2347,7 @@
     </row>
     <row r="64" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="12" t="s">
-        <v>121</v>
+        <v>150</v>
       </c>
       <c r="B64" s="12"/>
       <c r="C64" s="12"/>
@@ -2174,7 +2357,7 @@
     </row>
     <row r="65" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="12" t="s">
-        <v>122</v>
+        <v>151</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12"/>
@@ -2184,7 +2367,7 @@
     </row>
     <row r="66" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="12" t="s">
-        <v>123</v>
+        <v>152</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12"/>
@@ -2192,25 +2375,25 @@
       <c r="E66" s="12"/>
       <c r="F66" s="12"/>
     </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" s="16" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="B121" s="17" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="B122" s="17" t="s">
-        <v>128</v>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="16" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="B69" s="17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B70" s="17" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(contracts): reconcile catalog import persistence policy
</commit_message>
<xml_diff>
--- a/docs/catalog-import/catalog-import-v1-template.xlsx
+++ b/docs/catalog-import/catalog-import-v1-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="159">
   <si>
     <t>批次内关联 ID【必填】</t>
   </si>
@@ -238,7 +238,7 @@
     <t>纯 synthetic 示例：province=福建省，prefecture=泉州市，county=洛江区，currentLocation=万安某处，currentCustodian=某文物管理机构。该示例不是 production data。</t>
   </si>
   <si>
-    <t>SourceId mirroring：03_Provenance 可在相同 catalogImportId 下镜像主表 sourceId 以扩展同一 SourceRecord metadata；重复 pair 或跨 Catalog 绑定冲突会失败。</t>
+    <t>SourceId persistence：每条 01_Catalog 在 Apply 时都需要一条相同 catalogImportId + sourceId 的 03_Provenance 主来源行；可另加其他来源。重复 pair 或跨 Catalog 绑定冲突会失败。</t>
   </si>
   <si>
     <t>C. Field Guide</t>
@@ -394,7 +394,7 @@
     <t>blank 不删除；CLEAR 会进入逐字段审批。</t>
   </si>
   <si>
-    <t>仅供 Owner 审核；不发布，不提供 destructive state。</t>
+    <t>仅供 Owner 审核；不发布。当前 supplied ownerNote 会 fail closed，不发生 Apply 写入。</t>
   </si>
   <si>
     <t>纯合成内部备注</t>
@@ -460,10 +460,13 @@
     <t>D. Advanced persistence / approval / hash notes</t>
   </si>
   <si>
-    <t>当前 Apply 有硬性 persistence-gap gate：temporal/region/location/custodian、aliasType、SourceRecord/provenance 与 durable Import Batch audit 未闭合前不得无损 Apply。Approval 不能授权 silent loss。</t>
-  </si>
-  <si>
-    <t>Alias row 受 ALIAS_TYPE_STORAGE_REQUIRED 阻断；raw provenance 受 PROVENANCE_STORAGE_REQUIRED 阻断。不得部分写入或用 audit preservation 冒充 domain persistence。</t>
+    <t>当前 Apply 已支持：title / CatalogKind、事实字段 value/state、description、alias / aliasType、SourceId / provenance metadata，以及 durable Import Batch audit。</t>
+  </si>
+  <si>
+    <t>仍然 fail closed：supplied ownerNote 不会静默丢弃；alias collection UPDATE 的 replace / merge / delete semantics 尚未定义。</t>
+  </si>
+  <si>
+    <t>Research evidence、Owner research decisions/state 与 external ResearchRecord / SQLite state 不属于 catalog-import/v1。</t>
   </si>
   <si>
     <t>Identity conflict 始终不可 approval；Level A/B critical changes 需要 field-level approval；每个 CLEAR 都需要 field-level approval。</t>
@@ -2375,29 +2378,39 @@
       <c r="E66" s="12"/>
       <c r="F66" s="12"/>
     </row>
+    <row r="67" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B67" s="12"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12"/>
+    </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="16" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
@@ -2424,6 +2437,7 @@
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A65:F65"/>
     <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A67:F67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
fix(contracts): reconcile catalog import persistence policy (#36)
Co-authored-by: jj3445 <jj3445@columbia.edu>
</commit_message>
<xml_diff>
--- a/docs/catalog-import/catalog-import-v1-template.xlsx
+++ b/docs/catalog-import/catalog-import-v1-template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="159">
   <si>
     <t>批次内关联 ID【必填】</t>
   </si>
@@ -238,7 +238,7 @@
     <t>纯 synthetic 示例：province=福建省，prefecture=泉州市，county=洛江区，currentLocation=万安某处，currentCustodian=某文物管理机构。该示例不是 production data。</t>
   </si>
   <si>
-    <t>SourceId mirroring：03_Provenance 可在相同 catalogImportId 下镜像主表 sourceId 以扩展同一 SourceRecord metadata；重复 pair 或跨 Catalog 绑定冲突会失败。</t>
+    <t>SourceId persistence：每条 01_Catalog 在 Apply 时都需要一条相同 catalogImportId + sourceId 的 03_Provenance 主来源行；可另加其他来源。重复 pair 或跨 Catalog 绑定冲突会失败。</t>
   </si>
   <si>
     <t>C. Field Guide</t>
@@ -394,7 +394,7 @@
     <t>blank 不删除；CLEAR 会进入逐字段审批。</t>
   </si>
   <si>
-    <t>仅供 Owner 审核；不发布，不提供 destructive state。</t>
+    <t>仅供 Owner 审核；不发布。当前 supplied ownerNote 会 fail closed，不发生 Apply 写入。</t>
   </si>
   <si>
     <t>纯合成内部备注</t>
@@ -460,10 +460,13 @@
     <t>D. Advanced persistence / approval / hash notes</t>
   </si>
   <si>
-    <t>当前 Apply 有硬性 persistence-gap gate：temporal/region/location/custodian、aliasType、SourceRecord/provenance 与 durable Import Batch audit 未闭合前不得无损 Apply。Approval 不能授权 silent loss。</t>
-  </si>
-  <si>
-    <t>Alias row 受 ALIAS_TYPE_STORAGE_REQUIRED 阻断；raw provenance 受 PROVENANCE_STORAGE_REQUIRED 阻断。不得部分写入或用 audit preservation 冒充 domain persistence。</t>
+    <t>当前 Apply 已支持：title / CatalogKind、事实字段 value/state、description、alias / aliasType、SourceId / provenance metadata，以及 durable Import Batch audit。</t>
+  </si>
+  <si>
+    <t>仍然 fail closed：supplied ownerNote 不会静默丢弃；alias collection UPDATE 的 replace / merge / delete semantics 尚未定义。</t>
+  </si>
+  <si>
+    <t>Research evidence、Owner research decisions/state 与 external ResearchRecord / SQLite state 不属于 catalog-import/v1。</t>
   </si>
   <si>
     <t>Identity conflict 始终不可 approval；Level A/B critical changes 需要 field-level approval；每个 CLEAR 都需要 field-level approval。</t>
@@ -2375,29 +2378,39 @@
       <c r="E66" s="12"/>
       <c r="F66" s="12"/>
     </row>
+    <row r="67" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B67" s="12"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12"/>
+    </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" s="16" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="27">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
@@ -2424,6 +2437,7 @@
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A65:F65"/>
     <mergeCell ref="A66:F66"/>
+    <mergeCell ref="A67:F67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>